<commit_message>
Online Safety Bill: sort the register's Summary sheet by incident id
Michael's edit, made in Excel on 2026-09-12 and held in a stash while the
corpus work was on another branch. The Summary sheet now lists incidents
in id order rather than by severity, with ids zero-padded (#01 to #20) so
that they sort correctly as text. The Incidents sheet keeps unpadded ids
(#1 to #20), matching NOTES.md, the reports and the module comments.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/subjects/new-zealand/online-safety-minimum-age-bill-2026/registers/incident-register.xlsx
+++ b/subjects/new-zealand/online-safety-minimum-age-bill-2026/registers/incident-register.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="243">
   <si>
     <t xml:space="preserve">Online Safety (Minimum Age and Child Safety Risk Assessment) Bill 2026 No 339-1</t>
   </si>
@@ -139,334 +139,364 @@
     <t xml:space="preserve">Category</t>
   </si>
   <si>
+    <t xml:space="preserve">#01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excluded-service carve-out attaches only to limb (a)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scope gap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A broadcast-only feed with every risky feature falls outside clause 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Under-inclusion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The excluded-service carve-out is available by restructuring, and is indifferent to features</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One engagement-metric feature pulls ordinary publishing and repository services into scope</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tier partition over specified liability acts - verified, no defect</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consistency check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A section 7 designation displaces the company that actually runs the platform</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liability gap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Designation power cannot reach a controller outside both limbs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exemption route reaches regulation-added platforms - verified, no defect</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The minimum age duty states only which methods fail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Definitional openness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A duty with no time for performance carries Tier 2 liability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deadline omission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The only duty binding the regulator carries no consequence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unenforceable duty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Significant change' is defined inclusively</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The regulator is the chief executive of the department that wrote the Bill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Structural</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breach of an enforceable undertaking is not a specified liability act</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enforcement gap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The measure with immediate public effect carries the least process</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Procedural asymmetry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The only imprisonable offence is switched off by a lesser civil breach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exemption from any or all requirements of the Act by Order in Council</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delegated power</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A prohibition with no consequence, defined by the weakest regulation-making power</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transitional relief goes to the paperwork duty, not the duty affecting users</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transitional gap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The scope test is self-executing and there is no register of age-restricted platforms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clauses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consequence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Related</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raised</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
     <t xml:space="preserve">#1</t>
   </si>
   <si>
-    <t xml:space="preserve">Excluded-service carve-out attaches only to limb (a)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scope gap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High</t>
+    <t xml:space="preserve">cl 5(1)(b), cl 5(2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cl 5(2) defines 'excluded service' and cl 5(1)(a)(iv) requires that a service is not one. cl 5(1)(b), the AI companion limb, carries no such carve-out and requires no specified feature.
+Buddy.ai uses AI primarily to form a personal connection to the user, but the primary service of the internet service itself is to educate.  But there is no exclusion for the AI-compaign limb.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A service that solely or primarily enables healthcare or education - and so is excluded from limb (a) - is caught by limb (b) if it uses AI to simulate a personal connection. A therapy or tutoring chatbot falls out of scope and straight back in.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">part-1-preliminary.l4: #ASSERT 'the service is an age-restricted platform under section 5(1)(a)' 'a therapy chatbot' EQUALS FALSE; same fixture under 5(1)(b) EQUALS TRUE.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Machine-evaluated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">part-1-preliminary.l4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If intended, under-signposted; if not, a gap.</t>
   </si>
   <si>
     <t xml:space="preserve">#2</t>
   </si>
   <si>
-    <t xml:space="preserve">A broadcast-only feed with every risky feature falls outside clause 5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Under-inclusion</t>
+    <t xml:space="preserve">cl 5(1)(a)(ii), cl 5(1)(b)(iii)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cl 5(1)(a)(ii) requires that the service enables the exchange of digital content between 2 or more users. A service that publishes operator-generated or licensed content to a personalised, endless, time-limited feed, with no posting, commenting or messaging, satisfies every other element of limb (a) but not that one. Limb (b) does not reach it either: its AI recommends content, it does not simulate a personal connection.
+Vibes by Meta will fall through this loophole.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Bill's own account of risk - cl 5(2) specified features, and the cl 14(2)(b) matters about recommender systems, behaviour profiling and business model - is fully present, and the service is out of scope. As AI-generated feeds displace user-generated ones this becomes the ordinary case rather than an edge case. cl 62(1)(a) can specify such a service by regulation, but only one at a time and only after the Minister has considered, sought advice and consulted.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">part-1-preliminary.l4: on 'a broadcast-only recommender feed', #ASSERT 'the service has 1 or more specified features' EQUALS TRUE and #ASSERT 'the service is an age-restricted platform' EQUALS FALSE.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The exchange requirement is doing the work of a proxy for risk, and no longer tracks it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cl 5(2) excluded service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cl 5(2) excludes a service that 'solely or primarily' enables one of eight activities 'regardless of whether it meets the criteria in subsection (1)(a)(ii) and (iii)'. The carve-out is expressly indifferent to the specified features, so a service carrying all of them is excluded if its primary character falls within a listed activity.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primary character is a matter of degree that the operator largely controls through product design and marketing. A social feed restructured so that gaming predominates is outside limb (a) with its recommender, endless feed and disappearing posts intact. The same route runs through messaging, music and the cl 62(1)(c) regulation-made activity.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">part-1-preliminary.l4: on 'a social app wrapped in a game', #ASSERT 'the service has 1 or more specified features' EQUALS TRUE and #ASSERT 'the service is an age-restricted platform' EQUALS FALSE.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compare cl 5(1)(b), which has no carve-out at all - the two limbs are calibrated oppositely.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cl 5(2)(c), cl 5(1)(a)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cl 5(2)(c) makes it a specified feature to display 'information to a user about how others have viewed or engaged with the user's digital content or account'. A scholarly repository that shows authors their download and view counts has that feature, enables exchange between users (authors upload, readers download), and is accessible in New Zealand.
+SSRN would be age-restructed or geo-blocked preventing teenage prodigies from reading academic papers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whether such a service escapes turns entirely on whether it is characterised as solely or primarily an education service under cl 5(2)(f) - a question the Bill does not settle and which flips the outcome. The same analysis reaches academic repositories, preprint servers, code hosting with stars and view counts, and photo or writing communities. The consequence for a 15-year-old is no account, not no access, but for a repository whose downloads require an account the distinction collapses.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">part-1-preliminary.l4: 'a scholarly research repository' EQUALS TRUE and 'a scholarly repository read as education' EQUALS FALSE for 'the service is an age-restricted platform' - the same service, opposite results, on a characterisation the Bill leaves open.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raised from a reviewer scenario (SSRN) on 2026-09-11.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cl 34(3)(a)-(i), cll 45-47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cll 45-47 route cl 34(3)(a)-(c) to Tier 1, (d)-(g) to Tier 2, and (h)-(i) to Tier 3. The partition appears total and disjoint on its face but has not been machine-checked.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None on the text as drafted. The partition is total and disjoint. Recorded because it is prospective cover: if a paragraph is added to cl 34(3) without amending cll 45-47, the encoding fails to typecheck rather than leaving the new act unpenalised.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">part-3-subpart-3-remedies.l4: `the tier for` is a total function over the specified liability act enum; nine #ASSERT directives pin each act to its tier. All nine hold.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verified - no defect</t>
+  </si>
+  <si>
+    <t xml:space="preserve">part-3-subpart-3-remedies.l4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Negative result, retained as evidence of coverage.</t>
   </si>
   <si>
     <t xml:space="preserve">#6</t>
   </si>
   <si>
-    <t xml:space="preserve">A section 7 designation displaces the company that actually runs the platform</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Liability gap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A duty with no time for performance carries Tier 2 liability</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deadline omission</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The only imprisonable offence is switched off by a lesser civil breach</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enforcement gap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exemption from any or all requirements of the Act by Order in Council</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delegated power</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The scope test is self-executing and there is no register of age-restricted platforms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Structural</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The excluded-service carve-out is available by restructuring, and is indifferent to features</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One engagement-metric feature pulls ordinary publishing and repository services into scope</t>
+    <t xml:space="preserve">cl 6(1), cl 6(2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cl 6(2) provides that a designated person is 'the only operator ... while the designation is in place'. A person who manages or controls the platform's operations in New Zealand, and so is an operator under cl 6(1), ceases to be the operator once someone else is designated.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every Part 2 duty attaches to 'an operator of an age-restricted platform', so the displaced controller owes none while the designation stands. The Bill does not say what becomes of duties that accrued before the designation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">part-1-preliminary.l4: on 'a displaced controller', #ASSERT 'the person is an operator under section 6(1)' EQUALS TRUE and #ASSERT 'the person is the operator of the platform' EQUALS FALSE.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consider a savings provision for accrued duties.</t>
   </si>
   <si>
     <t xml:space="preserve">#7</t>
   </si>
   <si>
-    <t xml:space="preserve">Designation power cannot reach a controller outside both limbs</t>
+    <t xml:space="preserve">cl 7(1)(a), cl 7(1)(b)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cl 7(1) permits the regulator to designate only a cl 6(1) operator or an interconnected body corporate of one. No other person can be designated, however clearly they direct the platform.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cl 7(2)(a) gives the purpose of the power as providing certainty about who is and is not an operator. That certainty is unavailable in precisely the case where identifying the operator is hardest - a platform whose controller answers neither limb.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surfaced while encoding cl 7(1) in part-1-preliminary.l4; follows from the text of the limbs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reasoned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cl 19(3)(b) solves the same problem three clauses later by requiring the notice to specify the date.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cl 5(1)(c), cl 61, cl 62</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Three routes bring a service into scope: the cl 5(1)(a) and (b) tests, cl 62 regulations under cl 5(1)(c), and cl 7 designation of an operator. cl 61 exemption orders are the route out.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None. cl 61(1)(a) exempts an operator of an age-restricted platform, and a service specified under cl 62(1)(a) is an age-restricted platform by force of cl 5(1)(c), so the exemption route reaches it. Encoding cl 62 did show that each limb of cl 62(1) carries its own satisfaction test - cl 62(4) for (a) and (b), cl 62(6) for (c) - and they are not interchangeable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">part-3-subpart-5-other.l4: #ASSERT shows a cl 62(1)(c) recommendation failing where only the cl 62(4) test is satisfied, and succeeding for a cl 62(1)(a) recommendation on that test.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">part-3-subpart-5-other.l4</t>
   </si>
   <si>
     <t xml:space="preserve">#9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The minimum age duty states only which methods fail</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Definitional openness</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'Significant change' is defined inclusively</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The regulator is the chief executive of the department that wrote the Bill</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Breach of an enforceable undertaking is not a specified liability act</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The measure with immediate public effect carries the least process</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Procedural asymmetry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A prohibition with no consequence, defined by the weakest regulation-making power</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unenforceable duty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transitional relief goes to the paperwork duty, not the duty affecting users</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transitional gap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The only duty binding the regulator carries no consequence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Low</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tier partition over specified liability acts - verified, no defect</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Consistency check</t>
-  </si>
-  <si>
-    <t xml:space="preserve">None</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exemption route reaches regulation-added platforms - verified, no defect</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clauses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Consequence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evidence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Module</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Related</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Raised</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cl 5(1)(b), cl 5(2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cl 5(2) defines 'excluded service' and cl 5(1)(a)(iv) requires that a service is not one. cl 5(1)(b), the AI companion limb, carries no such carve-out and requires no specified feature.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A service that solely or primarily enables healthcare or education - and so is excluded from limb (a) - is caught by limb (b) if it uses AI to simulate a personal connection. A therapy or tutoring chatbot falls out of scope and straight back in.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">part-1-preliminary.l4: #ASSERT 'the service is an age-restricted platform under section 5(1)(a)' 'a therapy chatbot' EQUALS FALSE; same fixture under 5(1)(b) EQUALS TRUE.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Machine-evaluated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">part-1-preliminary.l4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">If intended, under-signposted; if not, a gap.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cl 5(1)(a)(ii), cl 5(1)(b)(iii)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cl 5(1)(a)(ii) requires that the service enables the exchange of digital content between 2 or more users. A service that publishes operator-generated or licensed content to a personalised, endless, time-limited feed, with no posting, commenting or messaging, satisfies every other element of limb (a) but not that one. Limb (b) does not reach it either: its AI recommends content, it does not simulate a personal connection.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Bill's own account of risk - cl 5(2) specified features, and the cl 14(2)(b) matters about recommender systems, behaviour profiling and business model - is fully present, and the service is out of scope. As AI-generated feeds displace user-generated ones this becomes the ordinary case rather than an edge case. cl 62(1)(a) can specify such a service by regulation, but only one at a time and only after the Minister has considered, sought advice and consulted.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">part-1-preliminary.l4: on 'a broadcast-only recommender feed', #ASSERT 'the service has 1 or more specified features' EQUALS TRUE and #ASSERT 'the service is an age-restricted platform' EQUALS FALSE.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The exchange requirement is doing the work of a proxy for risk, and no longer tracks it.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cl 5(2) excluded service</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cl 5(2) excludes a service that 'solely or primarily' enables one of eight activities 'regardless of whether it meets the criteria in subsection (1)(a)(ii) and (iii)'. The carve-out is expressly indifferent to the specified features, so a service carrying all of them is excluded if its primary character falls within a listed activity.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Primary character is a matter of degree that the operator largely controls through product design and marketing. A social feed restructured so that gaming predominates is outside limb (a) with its recommender, endless feed and disappearing posts intact. The same route runs through messaging, music and the cl 62(1)(c) regulation-made activity.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">part-1-preliminary.l4: on 'a social app wrapped in a game', #ASSERT 'the service has 1 or more specified features' EQUALS TRUE and #ASSERT 'the service is an age-restricted platform' EQUALS FALSE.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compare cl 5(1)(b), which has no carve-out at all - the two limbs are calibrated oppositely.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cl 5(2)(c), cl 5(1)(a)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cl 5(2)(c) makes it a specified feature to display 'information to a user about how others have viewed or engaged with the user's digital content or account'. A scholarly repository that shows authors their download and view counts has that feature, enables exchange between users (authors upload, readers download), and is accessible in New Zealand.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Whether such a service escapes turns entirely on whether it is characterised as solely or primarily an education service under cl 5(2)(f) - a question the Bill does not settle and which flips the outcome. The same analysis reaches academic repositories, preprint servers, code hosting with stars and view counts, and photo or writing communities. The consequence for a 15-year-old is no account, not no access, but for a repository whose downloads require an account the distinction collapses.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">part-1-preliminary.l4: 'a scholarly research repository' EQUALS TRUE and 'a scholarly repository read as education' EQUALS FALSE for 'the service is an age-restricted platform' - the same service, opposite results, on a characterisation the Bill leaves open.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Raised from a reviewer scenario (SSRN) on 2026-09-11.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cl 34(3)(a)-(i), cll 45-47</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cll 45-47 route cl 34(3)(a)-(c) to Tier 1, (d)-(g) to Tier 2, and (h)-(i) to Tier 3. The partition appears total and disjoint on its face but has not been machine-checked.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">None on the text as drafted. The partition is total and disjoint. Recorded because it is prospective cover: if a paragraph is added to cl 34(3) without amending cll 45-47, the encoding fails to typecheck rather than leaving the new act unpenalised.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">part-3-subpart-3-remedies.l4: `the tier for` is a total function over the specified liability act enum; nine #ASSERT directives pin each act to its tier. All nine hold.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verified - no defect</t>
-  </si>
-  <si>
-    <t xml:space="preserve">part-3-subpart-3-remedies.l4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Negative result, retained as evidence of coverage.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cl 6(1), cl 6(2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cl 6(2) provides that a designated person is 'the only operator ... while the designation is in place'. A person who manages or controls the platform's operations in New Zealand, and so is an operator under cl 6(1), ceases to be the operator once someone else is designated.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Every Part 2 duty attaches to 'an operator of an age-restricted platform', so the displaced controller owes none while the designation stands. The Bill does not say what becomes of duties that accrued before the designation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">part-1-preliminary.l4: on 'a displaced controller', #ASSERT 'the person is an operator under section 6(1)' EQUALS TRUE and #ASSERT 'the person is the operator of the platform' EQUALS FALSE.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Consider a savings provision for accrued duties.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cl 7(1)(a), cl 7(1)(b)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cl 7(1) permits the regulator to designate only a cl 6(1) operator or an interconnected body corporate of one. No other person can be designated, however clearly they direct the platform.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cl 7(2)(a) gives the purpose of the power as providing certainty about who is and is not an operator. That certainty is unavailable in precisely the case where identifying the operator is hardest - a platform whose controller answers neither limb.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Surfaced while encoding cl 7(1) in part-1-preliminary.l4; follows from the text of the limbs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reasoned</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cl 19(3)(b) solves the same problem three clauses later by requiring the notice to specify the date.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cl 5(1)(c), cl 61, cl 62</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Three routes bring a service into scope: the cl 5(1)(a) and (b) tests, cl 62 regulations under cl 5(1)(c), and cl 7 designation of an operator. cl 61 exemption orders are the route out.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">None. cl 61(1)(a) exempts an operator of an age-restricted platform, and a service specified under cl 62(1)(a) is an age-restricted platform by force of cl 5(1)(c), so the exemption route reaches it. Encoding cl 62 did show that each limb of cl 62(1) carries its own satisfaction test - cl 62(4) for (a) and (b), cl 62(6) for (c) - and they are not interchangeable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">part-3-subpart-5-other.l4: #ASSERT shows a cl 62(1)(c) recommendation failing where only the cl 62(4) test is satisfied, and succeeding for a cl 62(1)(a) recommendation on that test.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">part-3-subpart-5-other.l4</t>
   </si>
   <si>
     <t xml:space="preserve">cl 11(1), cl 11(2), cl 11(3)</t>
@@ -837,14 +867,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAF3EA"/>
-        <bgColor rgb="FFF2F2F2"/>
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFEAF3EA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFEAF3EA"/>
+        <fgColor rgb="FFEAF3EA"/>
+        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -897,120 +927,112 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1023,11 +1045,27 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF1F3864"/>
+          <fgColor rgb="FFEAF3EA"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE4E4"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1043,6 +1081,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF1F3864"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1491,10 +1537,10 @@
   <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="80"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="77.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1521,7 +1567,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
         <v>37</v>
       </c>
@@ -1535,7 +1581,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
         <v>41</v>
       </c>
@@ -1549,49 +1595,49 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
+    <row r="7" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D7" s="11" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="11" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+      <c r="B9" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="C9" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="D9" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="D9" s="11" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="10" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
         <v>53</v>
       </c>
@@ -1605,200 +1651,200 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
+    <row r="11" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="B12" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" s="11" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="D12" s="13" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
+    <row r="15" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="B15" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C16" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="B13" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="C15" s="13" t="s">
+      <c r="D16" s="13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="D21" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="D15" s="13" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>72</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="B18" s="13" t="s">
+      <c r="D22" s="13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="18.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C24" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="C18" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="D18" s="13" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="D19" s="13" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="B20" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="C20" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="D20" s="13" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="B21" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="D21" s="13" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="C22" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="D22" s="15" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="B23" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="C23" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="D23" s="17" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="B24" s="17" t="s">
-        <v>92</v>
-      </c>
-      <c r="C24" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="D24" s="17" t="s">
-        <v>90</v>
+      <c r="D24" s="11" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -1881,10 +1927,10 @@
     </row>
     <row r="2" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="19" t="s">
-        <v>37</v>
+        <v>102</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C2" s="20" t="s">
         <v>38</v>
@@ -1893,16 +1939,16 @@
         <v>39</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I2" s="20" t="s">
         <v>40</v>
@@ -1911,22 +1957,22 @@
         <v>18</v>
       </c>
       <c r="K2" s="20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L2" s="20"/>
       <c r="M2" s="20" t="s">
         <v>9</v>
       </c>
       <c r="N2" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="19" t="s">
-        <v>41</v>
+        <v>110</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C3" s="20" t="s">
         <v>42</v>
@@ -1935,16 +1981,16 @@
         <v>43</v>
       </c>
       <c r="E3" s="20" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="G3" s="20" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="H3" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I3" s="20" t="s">
         <v>40</v>
@@ -1953,172 +1999,172 @@
         <v>18</v>
       </c>
       <c r="K3" s="20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L3" s="20" t="s">
-        <v>37</v>
+        <v>102</v>
       </c>
       <c r="M3" s="20" t="s">
         <v>9</v>
       </c>
       <c r="N3" s="20" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>59</v>
+        <v>116</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>43</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="F4" s="20" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="G4" s="20" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I4" s="20" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="J4" s="20" t="s">
         <v>18</v>
       </c>
       <c r="K4" s="20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L4" s="20" t="s">
-        <v>37</v>
+        <v>102</v>
       </c>
       <c r="M4" s="20" t="s">
         <v>9</v>
       </c>
       <c r="N4" s="20" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>62</v>
+        <v>122</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="D5" s="20" t="s">
         <v>39</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I5" s="20" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="J5" s="20" t="s">
         <v>18</v>
       </c>
       <c r="K5" s="20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L5" s="20" t="s">
-        <v>37</v>
+        <v>102</v>
       </c>
       <c r="M5" s="20" t="s">
         <v>9</v>
       </c>
       <c r="N5" s="20" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>87</v>
+        <v>128</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>88</v>
+        <v>50</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>89</v>
+        <v>51</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="G6" s="20" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="H6" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I6" s="20" t="s">
-        <v>90</v>
+        <v>52</v>
       </c>
       <c r="J6" s="20" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="K6" s="20" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="L6" s="20"/>
       <c r="M6" s="20" t="s">
         <v>9</v>
       </c>
       <c r="N6" s="20" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>44</v>
+        <v>136</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I7" s="20" t="s">
         <v>40</v>
@@ -2127,168 +2173,168 @@
         <v>18</v>
       </c>
       <c r="K7" s="20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L7" s="20"/>
       <c r="M7" s="20" t="s">
         <v>9</v>
       </c>
       <c r="N7" s="20" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>64</v>
+        <v>142</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="D8" s="20" t="s">
         <v>39</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="G8" s="20" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="I8" s="20" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="J8" s="20" t="s">
         <v>18</v>
       </c>
       <c r="K8" s="20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L8" s="20" t="s">
-        <v>44</v>
+        <v>136</v>
       </c>
       <c r="M8" s="20" t="s">
         <v>9</v>
       </c>
       <c r="N8" s="20" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>91</v>
+        <v>149</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>92</v>
+        <v>59</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>89</v>
+        <v>51</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="G9" s="20" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="H9" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I9" s="20" t="s">
-        <v>90</v>
+        <v>52</v>
       </c>
       <c r="J9" s="20" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="K9" s="20" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="L9" s="20"/>
       <c r="M9" s="20" t="s">
         <v>9</v>
       </c>
       <c r="N9" s="20" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>66</v>
+        <v>155</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="G10" s="20" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="H10" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I10" s="20" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="J10" s="20" t="s">
         <v>18</v>
       </c>
       <c r="K10" s="20" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="L10" s="20"/>
       <c r="M10" s="20" t="s">
         <v>9</v>
       </c>
       <c r="N10" s="20" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="G11" s="20" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="H11" s="20" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="I11" s="20" t="s">
         <v>40</v>
@@ -2297,91 +2343,91 @@
         <v>18</v>
       </c>
       <c r="K11" s="20" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="L11" s="20"/>
       <c r="M11" s="20" t="s">
         <v>9</v>
       </c>
       <c r="N11" s="20" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="E12" s="20" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="G12" s="20" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="H12" s="20" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="I12" s="20" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="J12" s="20" t="s">
         <v>18</v>
       </c>
       <c r="K12" s="20" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="L12" s="20"/>
       <c r="M12" s="20" t="s">
         <v>9</v>
       </c>
       <c r="N12" s="20" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="E13" s="20" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="G13" s="20" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="H13" s="20" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="I13" s="20" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="J13" s="20" t="s">
         <v>18</v>
       </c>
       <c r="K13" s="20" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="L13" s="20"/>
       <c r="M13" s="20" t="s">
@@ -2391,121 +2437,121 @@
     </row>
     <row r="14" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="J14" s="13" t="s">
         <v>22</v>
       </c>
       <c r="K14" s="13" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="L14" s="13"/>
       <c r="M14" s="13" t="s">
         <v>9</v>
       </c>
       <c r="N14" s="13" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>52</v>
+        <v>77</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="F15" s="20" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="G15" s="20" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="H15" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I15" s="20" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="J15" s="20" t="s">
         <v>18</v>
       </c>
       <c r="K15" s="20" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="L15" s="20"/>
       <c r="M15" s="20" t="s">
         <v>9</v>
       </c>
       <c r="N15" s="20" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="F16" s="20" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="G16" s="20" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="H16" s="20" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="I16" s="20" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="J16" s="20" t="s">
         <v>18</v>
       </c>
       <c r="K16" s="20" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="L16" s="20"/>
       <c r="M16" s="20" t="s">
@@ -2515,28 +2561,28 @@
     </row>
     <row r="17" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>50</v>
+        <v>81</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>51</v>
+        <v>82</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>52</v>
+        <v>77</v>
       </c>
       <c r="E17" s="20" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="F17" s="20" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="G17" s="20" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="H17" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I17" s="20" t="s">
         <v>40</v>
@@ -2545,40 +2591,40 @@
         <v>18</v>
       </c>
       <c r="K17" s="20" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="L17" s="20"/>
       <c r="M17" s="20" t="s">
         <v>9</v>
       </c>
       <c r="N17" s="20" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
-        <v>53</v>
+        <v>83</v>
       </c>
       <c r="B18" s="20" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>54</v>
+        <v>84</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="E18" s="20" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="F18" s="20" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="G18" s="20" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="H18" s="20" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="I18" s="20" t="s">
         <v>40</v>
@@ -2587,124 +2633,124 @@
         <v>18</v>
       </c>
       <c r="K18" s="20" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="L18" s="20"/>
       <c r="M18" s="20" t="s">
         <v>9</v>
       </c>
       <c r="N18" s="20" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="E19" s="20" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="F19" s="20" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="G19" s="20" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="H19" s="20" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="I19" s="20" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="J19" s="20" t="s">
         <v>18</v>
       </c>
       <c r="K19" s="20" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="L19" s="20"/>
       <c r="M19" s="20" t="s">
         <v>9</v>
       </c>
       <c r="N19" s="20" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="E20" s="20" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="F20" s="20" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="G20" s="20" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="H20" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I20" s="20" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="J20" s="20" t="s">
         <v>18</v>
       </c>
       <c r="K20" s="20" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="L20" s="20"/>
       <c r="M20" s="20" t="s">
         <v>9</v>
       </c>
       <c r="N20" s="20" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>56</v>
+        <v>91</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>57</v>
+        <v>92</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="E21" s="20" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="F21" s="20" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="G21" s="20" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="H21" s="20" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="I21" s="20" t="s">
         <v>40</v>
@@ -2713,14 +2759,14 @@
         <v>18</v>
       </c>
       <c r="K21" s="20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L21" s="20"/>
       <c r="M21" s="20" t="s">
         <v>9</v>
       </c>
       <c r="N21" s="20" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -2751,261 +2797,261 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="21" t="s">
-        <v>208</v>
+      <c r="A1" s="7" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="D3" s="22" t="s">
-        <v>209</v>
+      <c r="D3" s="9" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="21" t="s">
+        <v>219</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>220</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="D4" s="21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>222</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="D5" s="21" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="21" t="s">
+        <v>160</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>223</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="D6" s="21" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="21" t="s">
+        <v>179</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>224</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="D7" s="21" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>225</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="D8" s="21" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="21" t="s">
+        <v>134</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>226</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>227</v>
+      </c>
+      <c r="D9" s="21" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21" t="s">
+        <v>195</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>228</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="D10" s="21" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="s">
+        <v>154</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>229</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="D11" s="21" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="s">
         <v>210</v>
       </c>
-      <c r="B4" s="23" t="s">
-        <v>211</v>
-      </c>
-      <c r="C4" s="23" t="s">
-        <v>212</v>
-      </c>
-      <c r="D4" s="23" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="s">
-        <v>107</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>213</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>212</v>
-      </c>
-      <c r="D5" s="23" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
-        <v>151</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>214</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>212</v>
-      </c>
-      <c r="D6" s="23" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>215</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>212</v>
-      </c>
-      <c r="D7" s="23" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="23" t="s">
-        <v>176</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>216</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>212</v>
-      </c>
-      <c r="D8" s="23" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23" t="s">
-        <v>129</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>217</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>218</v>
-      </c>
-      <c r="D9" s="23" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="s">
-        <v>186</v>
-      </c>
-      <c r="B10" s="23" t="s">
-        <v>219</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>212</v>
-      </c>
-      <c r="D10" s="23" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23" t="s">
-        <v>146</v>
-      </c>
-      <c r="B11" s="23" t="s">
-        <v>220</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>212</v>
-      </c>
-      <c r="D11" s="23" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="23" t="s">
-        <v>201</v>
-      </c>
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="21" t="s">
+        <v>230</v>
+      </c>
+      <c r="C12" s="21" t="s">
         <v>221</v>
       </c>
-      <c r="C12" s="23" t="s">
-        <v>212</v>
-      </c>
-      <c r="D12" s="23" t="n">
+      <c r="D12" s="21" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="24" t="s">
-        <v>222</v>
-      </c>
-      <c r="B13" s="25"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="24" t="n">
+      <c r="A13" s="22" t="s">
+        <v>231</v>
+      </c>
+      <c r="B13" s="23"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="22" t="n">
         <f aca="false">SUM(D4:D12)</f>
         <v>74</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="26" t="s">
-        <v>223</v>
+      <c r="A15" s="24" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="27" t="s">
-        <v>224</v>
-      </c>
-      <c r="B16" s="28" t="n">
+      <c r="A16" s="25" t="s">
+        <v>233</v>
+      </c>
+      <c r="B16" s="26" t="n">
         <f aca="false">COUNTA(Incidents!A2:A21)</f>
         <v>20</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="B17" s="28" t="n">
+      <c r="A17" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="B17" s="26" t="n">
         <f aca="false">COUNTIF(Incidents!H2:H21,"Machine-evaluated")</f>
         <v>11</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="27" t="s">
-        <v>225</v>
-      </c>
-      <c r="B18" s="28" t="n">
+      <c r="A18" s="25" t="s">
+        <v>234</v>
+      </c>
+      <c r="B18" s="26" t="n">
         <f aca="false">COUNTIF(Incidents!H2:H21,"Reasoned")</f>
         <v>9</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="27" t="s">
-        <v>226</v>
-      </c>
-      <c r="B19" s="28" t="n">
+      <c r="A19" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="B19" s="26" t="n">
         <f aca="false">COUNTIF(Incidents!I2:I21,"High")</f>
         <v>7</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="27" t="s">
-        <v>227</v>
-      </c>
-      <c r="B20" s="28" t="n">
+      <c r="A20" s="25" t="s">
+        <v>236</v>
+      </c>
+      <c r="B20" s="26" t="n">
         <f aca="false">COUNTIF(Incidents!I2:I21,"Medium")</f>
         <v>10</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="27" t="s">
-        <v>228</v>
-      </c>
-      <c r="B21" s="28" t="n">
+      <c r="A21" s="25" t="s">
+        <v>237</v>
+      </c>
+      <c r="B21" s="26" t="n">
         <f aca="false">COUNTIF(Incidents!I2:I21,"Low")</f>
         <v>1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="27" t="s">
-        <v>229</v>
-      </c>
-      <c r="B22" s="28" t="n">
+      <c r="A22" s="25" t="s">
+        <v>238</v>
+      </c>
+      <c r="B22" s="26" t="n">
         <f aca="false">COUNTIF(Incidents!J2:J21,"Open")</f>
         <v>17</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="27" t="s">
-        <v>230</v>
-      </c>
-      <c r="B23" s="28" t="n">
+      <c r="A23" s="25" t="s">
+        <v>239</v>
+      </c>
+      <c r="B23" s="26" t="n">
         <f aca="false">COUNTIF(Incidents!J2:J21,"Not yet encoded")</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="27" t="s">
-        <v>231</v>
-      </c>
-      <c r="B24" s="28" t="n">
+      <c r="A24" s="25" t="s">
+        <v>240</v>
+      </c>
+      <c r="B24" s="26" t="n">
         <f aca="false">COUNTIF(Incidents!J2:J21,"Candidate")</f>
         <v>1</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="27" t="s">
-        <v>232</v>
-      </c>
-      <c r="B25" s="28" t="n">
+      <c r="A25" s="25" t="s">
+        <v>241</v>
+      </c>
+      <c r="B25" s="26" t="n">
         <f aca="false">COUNTIF(Incidents!J2:J21,"Resolved")</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="27" t="s">
-        <v>233</v>
-      </c>
-      <c r="B26" s="28" t="n">
+      <c r="A26" s="25" t="s">
+        <v>242</v>
+      </c>
+      <c r="B26" s="26" t="n">
         <f aca="false">COUNTIF(Incidents!J2:J21,"Verified - no defect")</f>
         <v>2</v>
       </c>

</xml_diff>